<commit_message>
fix: 0.47Ohm resistor identification
Signed-off-by: Luca Mazilescu <luca.mazilescu@protonmail.com>
</commit_message>
<xml_diff>
--- a/Manufacturing/bom.xlsx
+++ b/Manufacturing/bom.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="115">
   <si>
     <t>Comment</t>
   </si>
@@ -55,10 +55,13 @@
     <t>C3682423</t>
   </si>
   <si>
-    <t>0.47Ω</t>
+    <t>470mΩ</t>
   </si>
   <si>
     <t>R1_EP_DR</t>
+  </si>
+  <si>
+    <t>C2089071</t>
   </si>
   <si>
     <t>0.47uH/6.5A/13mΩ</t>
@@ -362,7 +365,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -374,13 +377,18 @@
       <name val="Helvetica Neue"/>
     </font>
     <font>
+      <sz val="15"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -396,6 +404,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="12"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="13"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -526,28 +540,28 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -571,6 +585,7 @@
       <rgbColor rgb="ffa5a5a5"/>
       <rgbColor rgb="ff3f3f3f"/>
       <rgbColor rgb="ffdbdbdb"/>
+      <rgbColor rgb="ffffffff"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -587,10 +602,10 @@
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="5E5E5E"/>
+        <a:srgbClr val="A7A7A7"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="D5D5D5"/>
+        <a:srgbClr val="535353"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="00A2FF"/>
@@ -767,11 +782,14 @@
     <a:spDef>
       <a:spPr>
         <a:solidFill>
-          <a:srgbClr val="000000"/>
+          <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -780,33 +798,33 @@
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="ctr" defTabSz="584200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
-          <a:lnSpc>
-            <a:spcPct val="100000"/>
-          </a:lnSpc>
-          <a:spcBef>
-            <a:spcPts val="0"/>
-          </a:spcBef>
-          <a:spcAft>
-            <a:spcPts val="0"/>
-          </a:spcAft>
-          <a:buClrTx/>
-          <a:buSzTx/>
-          <a:buFontTx/>
-          <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1200" u="none" kumimoji="0" normalizeH="0">
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:uFillTx/>
-            <a:latin typeface="Helvetica Neue Medium"/>
-            <a:ea typeface="Helvetica Neue Medium"/>
-            <a:cs typeface="Helvetica Neue Medium"/>
-            <a:sym typeface="Helvetica Neue Medium"/>
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1045,12 +1063,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
-            <a:srgbClr val="000000"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="400000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1331,7 +1349,7 @@
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="457200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
           <a:lnSpc>
             <a:spcPct val="100000"/>
           </a:lnSpc>
@@ -1670,28 +1688,30 @@
       <c r="C5" t="s" s="8">
         <v>6</v>
       </c>
-      <c r="D5" s="9"/>
+      <c r="D5" t="s" s="8">
+        <v>16</v>
+      </c>
     </row>
     <row r="6" ht="20.05" customHeight="1">
       <c r="A6" t="s" s="6">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s" s="7">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s" s="8">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s" s="8">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" ht="32.05" customHeight="1">
       <c r="A7" t="s" s="6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s" s="7">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s" s="8">
         <v>6</v>
@@ -1700,10 +1720,10 @@
     </row>
     <row r="8" ht="20.05" customHeight="1">
       <c r="A8" t="s" s="6">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s" s="7">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s" s="8">
         <v>6</v>
@@ -1712,24 +1732,24 @@
     </row>
     <row r="9" ht="44.05" customHeight="1">
       <c r="A9" t="s" s="6">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s" s="7">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s" s="8">
         <v>6</v>
       </c>
       <c r="D9" t="s" s="8">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" ht="32.05" customHeight="1">
       <c r="A10" t="s" s="6">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s" s="7">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s" s="8">
         <v>12</v>
@@ -1738,22 +1758,22 @@
     </row>
     <row r="11" ht="20.05" customHeight="1">
       <c r="A11" t="s" s="6">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s" s="7">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s" s="8">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D11" s="9"/>
     </row>
     <row r="12" ht="20.05" customHeight="1">
       <c r="A12" t="s" s="6">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s" s="7">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s" s="8">
         <v>6</v>
@@ -1762,10 +1782,10 @@
     </row>
     <row r="13" ht="20.05" customHeight="1">
       <c r="A13" t="s" s="6">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13" t="s" s="7">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s" s="8">
         <v>12</v>
@@ -1774,10 +1794,10 @@
     </row>
     <row r="14" ht="20.05" customHeight="1">
       <c r="A14" t="s" s="6">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B14" t="s" s="7">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s" s="8">
         <v>6</v>
@@ -1786,10 +1806,10 @@
     </row>
     <row r="15" ht="32.05" customHeight="1">
       <c r="A15" t="s" s="6">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s" s="7">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s" s="8">
         <v>12</v>
@@ -1798,52 +1818,52 @@
     </row>
     <row r="16" ht="80.05" customHeight="1">
       <c r="A16" t="s" s="6">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s" s="7">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s" s="8">
         <v>12</v>
       </c>
       <c r="D16" t="s" s="8">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" ht="20.05" customHeight="1">
       <c r="A17" t="s" s="6">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B17" t="s" s="7">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s" s="8">
         <v>6</v>
       </c>
       <c r="D17" t="s" s="8">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" ht="32.05" customHeight="1">
       <c r="A18" t="s" s="6">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18" t="s" s="7">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C18" t="s" s="8">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s" s="8">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" ht="20.05" customHeight="1">
       <c r="A19" t="s" s="6">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s" s="7">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C19" t="s" s="8">
         <v>12</v>
@@ -1852,10 +1872,10 @@
     </row>
     <row r="20" ht="20.05" customHeight="1">
       <c r="A20" t="s" s="6">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B20" t="s" s="7">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C20" t="s" s="8">
         <v>12</v>
@@ -1864,48 +1884,48 @@
     </row>
     <row r="21" ht="20.05" customHeight="1">
       <c r="A21" t="s" s="6">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B21" t="s" s="7">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C21" t="s" s="8">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D21" s="9"/>
     </row>
     <row r="22" ht="20.05" customHeight="1">
       <c r="A22" t="s" s="6">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B22" t="s" s="7">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C22" t="s" s="8">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D22" s="9"/>
     </row>
     <row r="23" ht="20.05" customHeight="1">
       <c r="A23" t="s" s="6">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s" s="7">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C23" t="s" s="8">
         <v>6</v>
       </c>
       <c r="D23" t="s" s="8">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" ht="32.05" customHeight="1">
       <c r="A24" t="s" s="6">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s" s="7">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C24" t="s" s="8">
         <v>12</v>
@@ -1914,10 +1934,10 @@
     </row>
     <row r="25" ht="20.05" customHeight="1">
       <c r="A25" t="s" s="6">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B25" t="s" s="7">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C25" t="s" s="8">
         <v>12</v>
@@ -1926,10 +1946,10 @@
     </row>
     <row r="26" ht="20.05" customHeight="1">
       <c r="A26" t="s" s="6">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B26" t="s" s="7">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C26" t="s" s="8">
         <v>6</v>
@@ -1938,183 +1958,183 @@
     </row>
     <row r="27" ht="20.05" customHeight="1">
       <c r="A27" t="s" s="6">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B27" t="s" s="7">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C27" t="s" s="8">
         <v>6</v>
       </c>
       <c r="D27" t="s" s="8">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" ht="20.05" customHeight="1">
       <c r="A28" t="s" s="6">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B28" t="s" s="7">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C28" t="s" s="8">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D28" s="9"/>
     </row>
     <row r="29" ht="32.05" customHeight="1">
       <c r="A29" t="s" s="6">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B29" t="s" s="7">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C29" t="s" s="8">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D29" s="9"/>
     </row>
     <row r="30" ht="20.05" customHeight="1">
       <c r="A30" t="s" s="6">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B30" t="s" s="7">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C30" t="s" s="8">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D30" s="9"/>
     </row>
     <row r="31" ht="32.05" customHeight="1">
       <c r="A31" t="s" s="6">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B31" t="s" s="7">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C31" t="s" s="8">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D31" s="9"/>
     </row>
     <row r="32" ht="20.05" customHeight="1">
       <c r="A32" t="s" s="6">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B32" t="s" s="7">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C32" t="s" s="8">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D32" s="9"/>
     </row>
     <row r="33" ht="20.05" customHeight="1">
       <c r="A33" t="s" s="6">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B33" t="s" s="7">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C33" t="s" s="8">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D33" s="9"/>
     </row>
     <row r="34" ht="20.05" customHeight="1">
       <c r="A34" t="s" s="6">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B34" t="s" s="7">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C34" t="s" s="8">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D34" s="9"/>
     </row>
     <row r="35" ht="20.05" customHeight="1">
       <c r="A35" t="s" s="6">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B35" t="s" s="7">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C35" t="s" s="8">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D35" s="9"/>
     </row>
     <row r="36" ht="20.05" customHeight="1">
       <c r="A36" t="s" s="6">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B36" t="s" s="7">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C36" t="s" s="8">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D36" s="9"/>
     </row>
     <row r="37" ht="20.05" customHeight="1">
       <c r="A37" t="s" s="6">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B37" t="s" s="7">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C37" t="s" s="8">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D37" s="9"/>
     </row>
     <row r="38" ht="32.05" customHeight="1">
       <c r="A38" t="s" s="6">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B38" t="s" s="7">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C38" t="s" s="8">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D38" s="9"/>
     </row>
     <row r="39" ht="20.05" customHeight="1">
       <c r="A39" t="s" s="6">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B39" t="s" s="7">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C39" t="s" s="8">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D39" s="9"/>
     </row>
     <row r="40" ht="32.05" customHeight="1">
       <c r="A40" t="s" s="6">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B40" t="s" s="7">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C40" t="s" s="8">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D40" s="9"/>
     </row>
     <row r="41" ht="20.05" customHeight="1">
       <c r="A41" t="s" s="6">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B41" t="s" s="7">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C41" t="s" s="8">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D41" s="9"/>
     </row>

</xml_diff>